<commit_message>
feat(templates): outer + vertical bordered data grid on rows 3+
Per request, the blank templates carry an outer frame + vertical column
dividers (A..last) across ~50 empty data rows (3-52) with no inner horizontal
lines — a clean fillable grid; title + header keep the originals' exact
styling. The same outer+vertical scheme is applied to the export writer so a
filled export matches the template.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/Kontraktor.xlsx
+++ b/assets/templates/Kontraktor.xlsx
@@ -127,7 +127,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -355,6 +355,43 @@
         <color rgb="FF000000"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -362,7 +399,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -501,6 +538,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -782,7 +822,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02310675-88CA-42A3-B15C-D77C2FD8680D}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.85546875" bestFit="1" customWidth="1"/>
@@ -853,6 +893,706 @@
         <v>12</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="48"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
+      <c r="L3" s="48"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="49"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="49"/>
+      <c r="F4" s="49"/>
+      <c r="G4" s="49"/>
+      <c r="H4" s="49"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="49"/>
+      <c r="K4" s="49"/>
+      <c r="L4" s="49"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="49"/>
+      <c r="B5" s="49"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="49"/>
+      <c r="I5" s="49"/>
+      <c r="J5" s="49"/>
+      <c r="K5" s="49"/>
+      <c r="L5" s="49"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="49"/>
+      <c r="B6" s="49"/>
+      <c r="C6" s="49"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="49"/>
+      <c r="F6" s="49"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="49"/>
+      <c r="I6" s="49"/>
+      <c r="J6" s="49"/>
+      <c r="K6" s="49"/>
+      <c r="L6" s="49"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="49"/>
+      <c r="B7" s="49"/>
+      <c r="C7" s="49"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="49"/>
+      <c r="F7" s="49"/>
+      <c r="G7" s="49"/>
+      <c r="H7" s="49"/>
+      <c r="I7" s="49"/>
+      <c r="J7" s="49"/>
+      <c r="K7" s="49"/>
+      <c r="L7" s="49"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="49"/>
+      <c r="B8" s="49"/>
+      <c r="C8" s="49"/>
+      <c r="D8" s="49"/>
+      <c r="E8" s="49"/>
+      <c r="F8" s="49"/>
+      <c r="G8" s="49"/>
+      <c r="H8" s="49"/>
+      <c r="I8" s="49"/>
+      <c r="J8" s="49"/>
+      <c r="K8" s="49"/>
+      <c r="L8" s="49"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="49"/>
+      <c r="B9" s="49"/>
+      <c r="C9" s="49"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="49"/>
+      <c r="F9" s="49"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="49"/>
+      <c r="I9" s="49"/>
+      <c r="J9" s="49"/>
+      <c r="K9" s="49"/>
+      <c r="L9" s="49"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="49"/>
+      <c r="B10" s="49"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="49"/>
+      <c r="L10" s="49"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="49"/>
+      <c r="B11" s="49"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="49"/>
+      <c r="F11" s="49"/>
+      <c r="G11" s="49"/>
+      <c r="H11" s="49"/>
+      <c r="I11" s="49"/>
+      <c r="J11" s="49"/>
+      <c r="K11" s="49"/>
+      <c r="L11" s="49"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="49"/>
+      <c r="B12" s="49"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="49"/>
+      <c r="F12" s="49"/>
+      <c r="G12" s="49"/>
+      <c r="H12" s="49"/>
+      <c r="I12" s="49"/>
+      <c r="J12" s="49"/>
+      <c r="K12" s="49"/>
+      <c r="L12" s="49"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="49"/>
+      <c r="B13" s="49"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="49"/>
+      <c r="F13" s="49"/>
+      <c r="G13" s="49"/>
+      <c r="H13" s="49"/>
+      <c r="I13" s="49"/>
+      <c r="J13" s="49"/>
+      <c r="K13" s="49"/>
+      <c r="L13" s="49"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="49"/>
+      <c r="B14" s="49"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="49"/>
+      <c r="F14" s="49"/>
+      <c r="G14" s="49"/>
+      <c r="H14" s="49"/>
+      <c r="I14" s="49"/>
+      <c r="J14" s="49"/>
+      <c r="K14" s="49"/>
+      <c r="L14" s="49"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="49"/>
+      <c r="B15" s="49"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="49"/>
+      <c r="F15" s="49"/>
+      <c r="G15" s="49"/>
+      <c r="H15" s="49"/>
+      <c r="I15" s="49"/>
+      <c r="J15" s="49"/>
+      <c r="K15" s="49"/>
+      <c r="L15" s="49"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="49"/>
+      <c r="B16" s="49"/>
+      <c r="C16" s="49"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="49"/>
+      <c r="F16" s="49"/>
+      <c r="G16" s="49"/>
+      <c r="H16" s="49"/>
+      <c r="I16" s="49"/>
+      <c r="J16" s="49"/>
+      <c r="K16" s="49"/>
+      <c r="L16" s="49"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="49"/>
+      <c r="B17" s="49"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="49"/>
+      <c r="G17" s="49"/>
+      <c r="H17" s="49"/>
+      <c r="I17" s="49"/>
+      <c r="J17" s="49"/>
+      <c r="K17" s="49"/>
+      <c r="L17" s="49"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="49"/>
+      <c r="B18" s="49"/>
+      <c r="C18" s="49"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="49"/>
+      <c r="F18" s="49"/>
+      <c r="G18" s="49"/>
+      <c r="H18" s="49"/>
+      <c r="I18" s="49"/>
+      <c r="J18" s="49"/>
+      <c r="K18" s="49"/>
+      <c r="L18" s="49"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="49"/>
+      <c r="B19" s="49"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="49"/>
+      <c r="E19" s="49"/>
+      <c r="F19" s="49"/>
+      <c r="G19" s="49"/>
+      <c r="H19" s="49"/>
+      <c r="I19" s="49"/>
+      <c r="J19" s="49"/>
+      <c r="K19" s="49"/>
+      <c r="L19" s="49"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="49"/>
+      <c r="B20" s="49"/>
+      <c r="C20" s="49"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="49"/>
+      <c r="F20" s="49"/>
+      <c r="G20" s="49"/>
+      <c r="H20" s="49"/>
+      <c r="I20" s="49"/>
+      <c r="J20" s="49"/>
+      <c r="K20" s="49"/>
+      <c r="L20" s="49"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="49"/>
+      <c r="B21" s="49"/>
+      <c r="C21" s="49"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="49"/>
+      <c r="F21" s="49"/>
+      <c r="G21" s="49"/>
+      <c r="H21" s="49"/>
+      <c r="I21" s="49"/>
+      <c r="J21" s="49"/>
+      <c r="K21" s="49"/>
+      <c r="L21" s="49"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="49"/>
+      <c r="B22" s="49"/>
+      <c r="C22" s="49"/>
+      <c r="D22" s="49"/>
+      <c r="E22" s="49"/>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49"/>
+      <c r="H22" s="49"/>
+      <c r="I22" s="49"/>
+      <c r="J22" s="49"/>
+      <c r="K22" s="49"/>
+      <c r="L22" s="49"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="49"/>
+      <c r="B23" s="49"/>
+      <c r="C23" s="49"/>
+      <c r="D23" s="49"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="49"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="49"/>
+      <c r="K23" s="49"/>
+      <c r="L23" s="49"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="49"/>
+      <c r="B24" s="49"/>
+      <c r="C24" s="49"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="49"/>
+      <c r="I24" s="49"/>
+      <c r="J24" s="49"/>
+      <c r="K24" s="49"/>
+      <c r="L24" s="49"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="49"/>
+      <c r="B25" s="49"/>
+      <c r="C25" s="49"/>
+      <c r="D25" s="49"/>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="49"/>
+      <c r="I25" s="49"/>
+      <c r="J25" s="49"/>
+      <c r="K25" s="49"/>
+      <c r="L25" s="49"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="49"/>
+      <c r="B26" s="49"/>
+      <c r="C26" s="49"/>
+      <c r="D26" s="49"/>
+      <c r="E26" s="49"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="49"/>
+      <c r="H26" s="49"/>
+      <c r="I26" s="49"/>
+      <c r="J26" s="49"/>
+      <c r="K26" s="49"/>
+      <c r="L26" s="49"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="49"/>
+      <c r="B27" s="49"/>
+      <c r="C27" s="49"/>
+      <c r="D27" s="49"/>
+      <c r="E27" s="49"/>
+      <c r="F27" s="49"/>
+      <c r="G27" s="49"/>
+      <c r="H27" s="49"/>
+      <c r="I27" s="49"/>
+      <c r="J27" s="49"/>
+      <c r="K27" s="49"/>
+      <c r="L27" s="49"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="49"/>
+      <c r="B28" s="49"/>
+      <c r="C28" s="49"/>
+      <c r="D28" s="49"/>
+      <c r="E28" s="49"/>
+      <c r="F28" s="49"/>
+      <c r="G28" s="49"/>
+      <c r="H28" s="49"/>
+      <c r="I28" s="49"/>
+      <c r="J28" s="49"/>
+      <c r="K28" s="49"/>
+      <c r="L28" s="49"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="49"/>
+      <c r="B29" s="49"/>
+      <c r="C29" s="49"/>
+      <c r="D29" s="49"/>
+      <c r="E29" s="49"/>
+      <c r="F29" s="49"/>
+      <c r="G29" s="49"/>
+      <c r="H29" s="49"/>
+      <c r="I29" s="49"/>
+      <c r="J29" s="49"/>
+      <c r="K29" s="49"/>
+      <c r="L29" s="49"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="49"/>
+      <c r="B30" s="49"/>
+      <c r="C30" s="49"/>
+      <c r="D30" s="49"/>
+      <c r="E30" s="49"/>
+      <c r="F30" s="49"/>
+      <c r="G30" s="49"/>
+      <c r="H30" s="49"/>
+      <c r="I30" s="49"/>
+      <c r="J30" s="49"/>
+      <c r="K30" s="49"/>
+      <c r="L30" s="49"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="49"/>
+      <c r="B31" s="49"/>
+      <c r="C31" s="49"/>
+      <c r="D31" s="49"/>
+      <c r="E31" s="49"/>
+      <c r="F31" s="49"/>
+      <c r="G31" s="49"/>
+      <c r="H31" s="49"/>
+      <c r="I31" s="49"/>
+      <c r="J31" s="49"/>
+      <c r="K31" s="49"/>
+      <c r="L31" s="49"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="49"/>
+      <c r="B32" s="49"/>
+      <c r="C32" s="49"/>
+      <c r="D32" s="49"/>
+      <c r="E32" s="49"/>
+      <c r="F32" s="49"/>
+      <c r="G32" s="49"/>
+      <c r="H32" s="49"/>
+      <c r="I32" s="49"/>
+      <c r="J32" s="49"/>
+      <c r="K32" s="49"/>
+      <c r="L32" s="49"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="49"/>
+      <c r="B33" s="49"/>
+      <c r="C33" s="49"/>
+      <c r="D33" s="49"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="49"/>
+      <c r="G33" s="49"/>
+      <c r="H33" s="49"/>
+      <c r="I33" s="49"/>
+      <c r="J33" s="49"/>
+      <c r="K33" s="49"/>
+      <c r="L33" s="49"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="49"/>
+      <c r="B34" s="49"/>
+      <c r="C34" s="49"/>
+      <c r="D34" s="49"/>
+      <c r="E34" s="49"/>
+      <c r="F34" s="49"/>
+      <c r="G34" s="49"/>
+      <c r="H34" s="49"/>
+      <c r="I34" s="49"/>
+      <c r="J34" s="49"/>
+      <c r="K34" s="49"/>
+      <c r="L34" s="49"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="49"/>
+      <c r="B35" s="49"/>
+      <c r="C35" s="49"/>
+      <c r="D35" s="49"/>
+      <c r="E35" s="49"/>
+      <c r="F35" s="49"/>
+      <c r="G35" s="49"/>
+      <c r="H35" s="49"/>
+      <c r="I35" s="49"/>
+      <c r="J35" s="49"/>
+      <c r="K35" s="49"/>
+      <c r="L35" s="49"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="49"/>
+      <c r="B36" s="49"/>
+      <c r="C36" s="49"/>
+      <c r="D36" s="49"/>
+      <c r="E36" s="49"/>
+      <c r="F36" s="49"/>
+      <c r="G36" s="49"/>
+      <c r="H36" s="49"/>
+      <c r="I36" s="49"/>
+      <c r="J36" s="49"/>
+      <c r="K36" s="49"/>
+      <c r="L36" s="49"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="49"/>
+      <c r="B37" s="49"/>
+      <c r="C37" s="49"/>
+      <c r="D37" s="49"/>
+      <c r="E37" s="49"/>
+      <c r="F37" s="49"/>
+      <c r="G37" s="49"/>
+      <c r="H37" s="49"/>
+      <c r="I37" s="49"/>
+      <c r="J37" s="49"/>
+      <c r="K37" s="49"/>
+      <c r="L37" s="49"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="49"/>
+      <c r="B38" s="49"/>
+      <c r="C38" s="49"/>
+      <c r="D38" s="49"/>
+      <c r="E38" s="49"/>
+      <c r="F38" s="49"/>
+      <c r="G38" s="49"/>
+      <c r="H38" s="49"/>
+      <c r="I38" s="49"/>
+      <c r="J38" s="49"/>
+      <c r="K38" s="49"/>
+      <c r="L38" s="49"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="49"/>
+      <c r="B39" s="49"/>
+      <c r="C39" s="49"/>
+      <c r="D39" s="49"/>
+      <c r="E39" s="49"/>
+      <c r="F39" s="49"/>
+      <c r="G39" s="49"/>
+      <c r="H39" s="49"/>
+      <c r="I39" s="49"/>
+      <c r="J39" s="49"/>
+      <c r="K39" s="49"/>
+      <c r="L39" s="49"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="49"/>
+      <c r="B40" s="49"/>
+      <c r="C40" s="49"/>
+      <c r="D40" s="49"/>
+      <c r="E40" s="49"/>
+      <c r="F40" s="49"/>
+      <c r="G40" s="49"/>
+      <c r="H40" s="49"/>
+      <c r="I40" s="49"/>
+      <c r="J40" s="49"/>
+      <c r="K40" s="49"/>
+      <c r="L40" s="49"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="49"/>
+      <c r="B41" s="49"/>
+      <c r="C41" s="49"/>
+      <c r="D41" s="49"/>
+      <c r="E41" s="49"/>
+      <c r="F41" s="49"/>
+      <c r="G41" s="49"/>
+      <c r="H41" s="49"/>
+      <c r="I41" s="49"/>
+      <c r="J41" s="49"/>
+      <c r="K41" s="49"/>
+      <c r="L41" s="49"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="49"/>
+      <c r="B42" s="49"/>
+      <c r="C42" s="49"/>
+      <c r="D42" s="49"/>
+      <c r="E42" s="49"/>
+      <c r="F42" s="49"/>
+      <c r="G42" s="49"/>
+      <c r="H42" s="49"/>
+      <c r="I42" s="49"/>
+      <c r="J42" s="49"/>
+      <c r="K42" s="49"/>
+      <c r="L42" s="49"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="49"/>
+      <c r="B43" s="49"/>
+      <c r="C43" s="49"/>
+      <c r="D43" s="49"/>
+      <c r="E43" s="49"/>
+      <c r="F43" s="49"/>
+      <c r="G43" s="49"/>
+      <c r="H43" s="49"/>
+      <c r="I43" s="49"/>
+      <c r="J43" s="49"/>
+      <c r="K43" s="49"/>
+      <c r="L43" s="49"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="49"/>
+      <c r="B44" s="49"/>
+      <c r="C44" s="49"/>
+      <c r="D44" s="49"/>
+      <c r="E44" s="49"/>
+      <c r="F44" s="49"/>
+      <c r="G44" s="49"/>
+      <c r="H44" s="49"/>
+      <c r="I44" s="49"/>
+      <c r="J44" s="49"/>
+      <c r="K44" s="49"/>
+      <c r="L44" s="49"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="49"/>
+      <c r="B45" s="49"/>
+      <c r="C45" s="49"/>
+      <c r="D45" s="49"/>
+      <c r="E45" s="49"/>
+      <c r="F45" s="49"/>
+      <c r="G45" s="49"/>
+      <c r="H45" s="49"/>
+      <c r="I45" s="49"/>
+      <c r="J45" s="49"/>
+      <c r="K45" s="49"/>
+      <c r="L45" s="49"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="49"/>
+      <c r="B46" s="49"/>
+      <c r="C46" s="49"/>
+      <c r="D46" s="49"/>
+      <c r="E46" s="49"/>
+      <c r="F46" s="49"/>
+      <c r="G46" s="49"/>
+      <c r="H46" s="49"/>
+      <c r="I46" s="49"/>
+      <c r="J46" s="49"/>
+      <c r="K46" s="49"/>
+      <c r="L46" s="49"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="49"/>
+      <c r="B47" s="49"/>
+      <c r="C47" s="49"/>
+      <c r="D47" s="49"/>
+      <c r="E47" s="49"/>
+      <c r="F47" s="49"/>
+      <c r="G47" s="49"/>
+      <c r="H47" s="49"/>
+      <c r="I47" s="49"/>
+      <c r="J47" s="49"/>
+      <c r="K47" s="49"/>
+      <c r="L47" s="49"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="49"/>
+      <c r="B48" s="49"/>
+      <c r="C48" s="49"/>
+      <c r="D48" s="49"/>
+      <c r="E48" s="49"/>
+      <c r="F48" s="49"/>
+      <c r="G48" s="49"/>
+      <c r="H48" s="49"/>
+      <c r="I48" s="49"/>
+      <c r="J48" s="49"/>
+      <c r="K48" s="49"/>
+      <c r="L48" s="49"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="49"/>
+      <c r="B49" s="49"/>
+      <c r="C49" s="49"/>
+      <c r="D49" s="49"/>
+      <c r="E49" s="49"/>
+      <c r="F49" s="49"/>
+      <c r="G49" s="49"/>
+      <c r="H49" s="49"/>
+      <c r="I49" s="49"/>
+      <c r="J49" s="49"/>
+      <c r="K49" s="49"/>
+      <c r="L49" s="49"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="49"/>
+      <c r="B50" s="49"/>
+      <c r="C50" s="49"/>
+      <c r="D50" s="49"/>
+      <c r="E50" s="49"/>
+      <c r="F50" s="49"/>
+      <c r="G50" s="49"/>
+      <c r="H50" s="49"/>
+      <c r="I50" s="49"/>
+      <c r="J50" s="49"/>
+      <c r="K50" s="49"/>
+      <c r="L50" s="49"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="49"/>
+      <c r="B51" s="49"/>
+      <c r="C51" s="49"/>
+      <c r="D51" s="49"/>
+      <c r="E51" s="49"/>
+      <c r="F51" s="49"/>
+      <c r="G51" s="49"/>
+      <c r="H51" s="49"/>
+      <c r="I51" s="49"/>
+      <c r="J51" s="49"/>
+      <c r="K51" s="49"/>
+      <c r="L51" s="49"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="50"/>
+      <c r="B52" s="50"/>
+      <c r="C52" s="50"/>
+      <c r="D52" s="50"/>
+      <c r="E52" s="50"/>
+      <c r="F52" s="50"/>
+      <c r="G52" s="50"/>
+      <c r="H52" s="50"/>
+      <c r="I52" s="50"/>
+      <c r="J52" s="50"/>
+      <c r="K52" s="50"/>
+      <c r="L52" s="50"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>

</xml_diff>

<commit_message>
feat(templates): full grid (outer + vertical + horizontal) on data rows
Per follow-up, add the horizontal lines too: data rows 3+ now form a complete
black grid (every cell bordered on all sides) across A..last column. Applied
to both the static blank templates (rows 3-52) and the export writer
(getAllBorders on the data range).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/Kontraktor.xlsx
+++ b/assets/templates/Kontraktor.xlsx
@@ -127,7 +127,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -367,28 +367,6 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -399,7 +377,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -539,8 +517,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -908,690 +884,690 @@
       <c r="L3" s="48"/>
     </row>
     <row r="4">
-      <c r="A4" s="49"/>
-      <c r="B4" s="49"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
-      <c r="H4" s="49"/>
-      <c r="I4" s="49"/>
-      <c r="J4" s="49"/>
-      <c r="K4" s="49"/>
-      <c r="L4" s="49"/>
+      <c r="A4" s="48"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
+      <c r="H4" s="48"/>
+      <c r="I4" s="48"/>
+      <c r="J4" s="48"/>
+      <c r="K4" s="48"/>
+      <c r="L4" s="48"/>
     </row>
     <row r="5">
-      <c r="A5" s="49"/>
-      <c r="B5" s="49"/>
-      <c r="C5" s="49"/>
-      <c r="D5" s="49"/>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="49"/>
-      <c r="I5" s="49"/>
-      <c r="J5" s="49"/>
-      <c r="K5" s="49"/>
-      <c r="L5" s="49"/>
+      <c r="A5" s="48"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="48"/>
+      <c r="G5" s="48"/>
+      <c r="H5" s="48"/>
+      <c r="I5" s="48"/>
+      <c r="J5" s="48"/>
+      <c r="K5" s="48"/>
+      <c r="L5" s="48"/>
     </row>
     <row r="6">
-      <c r="A6" s="49"/>
-      <c r="B6" s="49"/>
-      <c r="C6" s="49"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="49"/>
-      <c r="H6" s="49"/>
-      <c r="I6" s="49"/>
-      <c r="J6" s="49"/>
-      <c r="K6" s="49"/>
-      <c r="L6" s="49"/>
+      <c r="A6" s="48"/>
+      <c r="B6" s="48"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="H6" s="48"/>
+      <c r="I6" s="48"/>
+      <c r="J6" s="48"/>
+      <c r="K6" s="48"/>
+      <c r="L6" s="48"/>
     </row>
     <row r="7">
-      <c r="A7" s="49"/>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
-      <c r="G7" s="49"/>
-      <c r="H7" s="49"/>
-      <c r="I7" s="49"/>
-      <c r="J7" s="49"/>
-      <c r="K7" s="49"/>
-      <c r="L7" s="49"/>
+      <c r="A7" s="48"/>
+      <c r="B7" s="48"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="48"/>
+      <c r="E7" s="48"/>
+      <c r="F7" s="48"/>
+      <c r="G7" s="48"/>
+      <c r="H7" s="48"/>
+      <c r="I7" s="48"/>
+      <c r="J7" s="48"/>
+      <c r="K7" s="48"/>
+      <c r="L7" s="48"/>
     </row>
     <row r="8">
-      <c r="A8" s="49"/>
-      <c r="B8" s="49"/>
-      <c r="C8" s="49"/>
-      <c r="D8" s="49"/>
-      <c r="E8" s="49"/>
-      <c r="F8" s="49"/>
-      <c r="G8" s="49"/>
-      <c r="H8" s="49"/>
-      <c r="I8" s="49"/>
-      <c r="J8" s="49"/>
-      <c r="K8" s="49"/>
-      <c r="L8" s="49"/>
+      <c r="A8" s="48"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
+      <c r="E8" s="48"/>
+      <c r="F8" s="48"/>
+      <c r="G8" s="48"/>
+      <c r="H8" s="48"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="48"/>
+      <c r="K8" s="48"/>
+      <c r="L8" s="48"/>
     </row>
     <row r="9">
-      <c r="A9" s="49"/>
-      <c r="B9" s="49"/>
-      <c r="C9" s="49"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
-      <c r="F9" s="49"/>
-      <c r="G9" s="49"/>
-      <c r="H9" s="49"/>
-      <c r="I9" s="49"/>
-      <c r="J9" s="49"/>
-      <c r="K9" s="49"/>
-      <c r="L9" s="49"/>
+      <c r="A9" s="48"/>
+      <c r="B9" s="48"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="48"/>
+      <c r="F9" s="48"/>
+      <c r="G9" s="48"/>
+      <c r="H9" s="48"/>
+      <c r="I9" s="48"/>
+      <c r="J9" s="48"/>
+      <c r="K9" s="48"/>
+      <c r="L9" s="48"/>
     </row>
     <row r="10">
-      <c r="A10" s="49"/>
-      <c r="B10" s="49"/>
-      <c r="C10" s="49"/>
-      <c r="D10" s="49"/>
-      <c r="E10" s="49"/>
-      <c r="F10" s="49"/>
-      <c r="G10" s="49"/>
-      <c r="H10" s="49"/>
-      <c r="I10" s="49"/>
-      <c r="J10" s="49"/>
-      <c r="K10" s="49"/>
-      <c r="L10" s="49"/>
+      <c r="A10" s="48"/>
+      <c r="B10" s="48"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="48"/>
+      <c r="I10" s="48"/>
+      <c r="J10" s="48"/>
+      <c r="K10" s="48"/>
+      <c r="L10" s="48"/>
     </row>
     <row r="11">
-      <c r="A11" s="49"/>
-      <c r="B11" s="49"/>
-      <c r="C11" s="49"/>
-      <c r="D11" s="49"/>
-      <c r="E11" s="49"/>
-      <c r="F11" s="49"/>
-      <c r="G11" s="49"/>
-      <c r="H11" s="49"/>
-      <c r="I11" s="49"/>
-      <c r="J11" s="49"/>
-      <c r="K11" s="49"/>
-      <c r="L11" s="49"/>
+      <c r="A11" s="48"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="48"/>
+      <c r="F11" s="48"/>
+      <c r="G11" s="48"/>
+      <c r="H11" s="48"/>
+      <c r="I11" s="48"/>
+      <c r="J11" s="48"/>
+      <c r="K11" s="48"/>
+      <c r="L11" s="48"/>
     </row>
     <row r="12">
-      <c r="A12" s="49"/>
-      <c r="B12" s="49"/>
-      <c r="C12" s="49"/>
-      <c r="D12" s="49"/>
-      <c r="E12" s="49"/>
-      <c r="F12" s="49"/>
-      <c r="G12" s="49"/>
-      <c r="H12" s="49"/>
-      <c r="I12" s="49"/>
-      <c r="J12" s="49"/>
-      <c r="K12" s="49"/>
-      <c r="L12" s="49"/>
+      <c r="A12" s="48"/>
+      <c r="B12" s="48"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="48"/>
+      <c r="E12" s="48"/>
+      <c r="F12" s="48"/>
+      <c r="G12" s="48"/>
+      <c r="H12" s="48"/>
+      <c r="I12" s="48"/>
+      <c r="J12" s="48"/>
+      <c r="K12" s="48"/>
+      <c r="L12" s="48"/>
     </row>
     <row r="13">
-      <c r="A13" s="49"/>
-      <c r="B13" s="49"/>
-      <c r="C13" s="49"/>
-      <c r="D13" s="49"/>
-      <c r="E13" s="49"/>
-      <c r="F13" s="49"/>
-      <c r="G13" s="49"/>
-      <c r="H13" s="49"/>
-      <c r="I13" s="49"/>
-      <c r="J13" s="49"/>
-      <c r="K13" s="49"/>
-      <c r="L13" s="49"/>
+      <c r="A13" s="48"/>
+      <c r="B13" s="48"/>
+      <c r="C13" s="48"/>
+      <c r="D13" s="48"/>
+      <c r="E13" s="48"/>
+      <c r="F13" s="48"/>
+      <c r="G13" s="48"/>
+      <c r="H13" s="48"/>
+      <c r="I13" s="48"/>
+      <c r="J13" s="48"/>
+      <c r="K13" s="48"/>
+      <c r="L13" s="48"/>
     </row>
     <row r="14">
-      <c r="A14" s="49"/>
-      <c r="B14" s="49"/>
-      <c r="C14" s="49"/>
-      <c r="D14" s="49"/>
-      <c r="E14" s="49"/>
-      <c r="F14" s="49"/>
-      <c r="G14" s="49"/>
-      <c r="H14" s="49"/>
-      <c r="I14" s="49"/>
-      <c r="J14" s="49"/>
-      <c r="K14" s="49"/>
-      <c r="L14" s="49"/>
+      <c r="A14" s="48"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
+      <c r="H14" s="48"/>
+      <c r="I14" s="48"/>
+      <c r="J14" s="48"/>
+      <c r="K14" s="48"/>
+      <c r="L14" s="48"/>
     </row>
     <row r="15">
-      <c r="A15" s="49"/>
-      <c r="B15" s="49"/>
-      <c r="C15" s="49"/>
-      <c r="D15" s="49"/>
-      <c r="E15" s="49"/>
-      <c r="F15" s="49"/>
-      <c r="G15" s="49"/>
-      <c r="H15" s="49"/>
-      <c r="I15" s="49"/>
-      <c r="J15" s="49"/>
-      <c r="K15" s="49"/>
-      <c r="L15" s="49"/>
+      <c r="A15" s="48"/>
+      <c r="B15" s="48"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="48"/>
+      <c r="E15" s="48"/>
+      <c r="F15" s="48"/>
+      <c r="G15" s="48"/>
+      <c r="H15" s="48"/>
+      <c r="I15" s="48"/>
+      <c r="J15" s="48"/>
+      <c r="K15" s="48"/>
+      <c r="L15" s="48"/>
     </row>
     <row r="16">
-      <c r="A16" s="49"/>
-      <c r="B16" s="49"/>
-      <c r="C16" s="49"/>
-      <c r="D16" s="49"/>
-      <c r="E16" s="49"/>
-      <c r="F16" s="49"/>
-      <c r="G16" s="49"/>
-      <c r="H16" s="49"/>
-      <c r="I16" s="49"/>
-      <c r="J16" s="49"/>
-      <c r="K16" s="49"/>
-      <c r="L16" s="49"/>
+      <c r="A16" s="48"/>
+      <c r="B16" s="48"/>
+      <c r="C16" s="48"/>
+      <c r="D16" s="48"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="48"/>
+      <c r="G16" s="48"/>
+      <c r="H16" s="48"/>
+      <c r="I16" s="48"/>
+      <c r="J16" s="48"/>
+      <c r="K16" s="48"/>
+      <c r="L16" s="48"/>
     </row>
     <row r="17">
-      <c r="A17" s="49"/>
-      <c r="B17" s="49"/>
-      <c r="C17" s="49"/>
-      <c r="D17" s="49"/>
-      <c r="E17" s="49"/>
-      <c r="F17" s="49"/>
-      <c r="G17" s="49"/>
-      <c r="H17" s="49"/>
-      <c r="I17" s="49"/>
-      <c r="J17" s="49"/>
-      <c r="K17" s="49"/>
-      <c r="L17" s="49"/>
+      <c r="A17" s="48"/>
+      <c r="B17" s="48"/>
+      <c r="C17" s="48"/>
+      <c r="D17" s="48"/>
+      <c r="E17" s="48"/>
+      <c r="F17" s="48"/>
+      <c r="G17" s="48"/>
+      <c r="H17" s="48"/>
+      <c r="I17" s="48"/>
+      <c r="J17" s="48"/>
+      <c r="K17" s="48"/>
+      <c r="L17" s="48"/>
     </row>
     <row r="18">
-      <c r="A18" s="49"/>
-      <c r="B18" s="49"/>
-      <c r="C18" s="49"/>
-      <c r="D18" s="49"/>
-      <c r="E18" s="49"/>
-      <c r="F18" s="49"/>
-      <c r="G18" s="49"/>
-      <c r="H18" s="49"/>
-      <c r="I18" s="49"/>
-      <c r="J18" s="49"/>
-      <c r="K18" s="49"/>
-      <c r="L18" s="49"/>
+      <c r="A18" s="48"/>
+      <c r="B18" s="48"/>
+      <c r="C18" s="48"/>
+      <c r="D18" s="48"/>
+      <c r="E18" s="48"/>
+      <c r="F18" s="48"/>
+      <c r="G18" s="48"/>
+      <c r="H18" s="48"/>
+      <c r="I18" s="48"/>
+      <c r="J18" s="48"/>
+      <c r="K18" s="48"/>
+      <c r="L18" s="48"/>
     </row>
     <row r="19">
-      <c r="A19" s="49"/>
-      <c r="B19" s="49"/>
-      <c r="C19" s="49"/>
-      <c r="D19" s="49"/>
-      <c r="E19" s="49"/>
-      <c r="F19" s="49"/>
-      <c r="G19" s="49"/>
-      <c r="H19" s="49"/>
-      <c r="I19" s="49"/>
-      <c r="J19" s="49"/>
-      <c r="K19" s="49"/>
-      <c r="L19" s="49"/>
+      <c r="A19" s="48"/>
+      <c r="B19" s="48"/>
+      <c r="C19" s="48"/>
+      <c r="D19" s="48"/>
+      <c r="E19" s="48"/>
+      <c r="F19" s="48"/>
+      <c r="G19" s="48"/>
+      <c r="H19" s="48"/>
+      <c r="I19" s="48"/>
+      <c r="J19" s="48"/>
+      <c r="K19" s="48"/>
+      <c r="L19" s="48"/>
     </row>
     <row r="20">
-      <c r="A20" s="49"/>
-      <c r="B20" s="49"/>
-      <c r="C20" s="49"/>
-      <c r="D20" s="49"/>
-      <c r="E20" s="49"/>
-      <c r="F20" s="49"/>
-      <c r="G20" s="49"/>
-      <c r="H20" s="49"/>
-      <c r="I20" s="49"/>
-      <c r="J20" s="49"/>
-      <c r="K20" s="49"/>
-      <c r="L20" s="49"/>
+      <c r="A20" s="48"/>
+      <c r="B20" s="48"/>
+      <c r="C20" s="48"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="48"/>
+      <c r="F20" s="48"/>
+      <c r="G20" s="48"/>
+      <c r="H20" s="48"/>
+      <c r="I20" s="48"/>
+      <c r="J20" s="48"/>
+      <c r="K20" s="48"/>
+      <c r="L20" s="48"/>
     </row>
     <row r="21">
-      <c r="A21" s="49"/>
-      <c r="B21" s="49"/>
-      <c r="C21" s="49"/>
-      <c r="D21" s="49"/>
-      <c r="E21" s="49"/>
-      <c r="F21" s="49"/>
-      <c r="G21" s="49"/>
-      <c r="H21" s="49"/>
-      <c r="I21" s="49"/>
-      <c r="J21" s="49"/>
-      <c r="K21" s="49"/>
-      <c r="L21" s="49"/>
+      <c r="A21" s="48"/>
+      <c r="B21" s="48"/>
+      <c r="C21" s="48"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="48"/>
+      <c r="F21" s="48"/>
+      <c r="G21" s="48"/>
+      <c r="H21" s="48"/>
+      <c r="I21" s="48"/>
+      <c r="J21" s="48"/>
+      <c r="K21" s="48"/>
+      <c r="L21" s="48"/>
     </row>
     <row r="22">
-      <c r="A22" s="49"/>
-      <c r="B22" s="49"/>
-      <c r="C22" s="49"/>
-      <c r="D22" s="49"/>
-      <c r="E22" s="49"/>
-      <c r="F22" s="49"/>
-      <c r="G22" s="49"/>
-      <c r="H22" s="49"/>
-      <c r="I22" s="49"/>
-      <c r="J22" s="49"/>
-      <c r="K22" s="49"/>
-      <c r="L22" s="49"/>
+      <c r="A22" s="48"/>
+      <c r="B22" s="48"/>
+      <c r="C22" s="48"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="48"/>
+      <c r="F22" s="48"/>
+      <c r="G22" s="48"/>
+      <c r="H22" s="48"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="48"/>
+      <c r="K22" s="48"/>
+      <c r="L22" s="48"/>
     </row>
     <row r="23">
-      <c r="A23" s="49"/>
-      <c r="B23" s="49"/>
-      <c r="C23" s="49"/>
-      <c r="D23" s="49"/>
-      <c r="E23" s="49"/>
-      <c r="F23" s="49"/>
-      <c r="G23" s="49"/>
-      <c r="H23" s="49"/>
-      <c r="I23" s="49"/>
-      <c r="J23" s="49"/>
-      <c r="K23" s="49"/>
-      <c r="L23" s="49"/>
+      <c r="A23" s="48"/>
+      <c r="B23" s="48"/>
+      <c r="C23" s="48"/>
+      <c r="D23" s="48"/>
+      <c r="E23" s="48"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="48"/>
+      <c r="H23" s="48"/>
+      <c r="I23" s="48"/>
+      <c r="J23" s="48"/>
+      <c r="K23" s="48"/>
+      <c r="L23" s="48"/>
     </row>
     <row r="24">
-      <c r="A24" s="49"/>
-      <c r="B24" s="49"/>
-      <c r="C24" s="49"/>
-      <c r="D24" s="49"/>
-      <c r="E24" s="49"/>
-      <c r="F24" s="49"/>
-      <c r="G24" s="49"/>
-      <c r="H24" s="49"/>
-      <c r="I24" s="49"/>
-      <c r="J24" s="49"/>
-      <c r="K24" s="49"/>
-      <c r="L24" s="49"/>
+      <c r="A24" s="48"/>
+      <c r="B24" s="48"/>
+      <c r="C24" s="48"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="48"/>
+      <c r="F24" s="48"/>
+      <c r="G24" s="48"/>
+      <c r="H24" s="48"/>
+      <c r="I24" s="48"/>
+      <c r="J24" s="48"/>
+      <c r="K24" s="48"/>
+      <c r="L24" s="48"/>
     </row>
     <row r="25">
-      <c r="A25" s="49"/>
-      <c r="B25" s="49"/>
-      <c r="C25" s="49"/>
-      <c r="D25" s="49"/>
-      <c r="E25" s="49"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="49"/>
-      <c r="H25" s="49"/>
-      <c r="I25" s="49"/>
-      <c r="J25" s="49"/>
-      <c r="K25" s="49"/>
-      <c r="L25" s="49"/>
+      <c r="A25" s="48"/>
+      <c r="B25" s="48"/>
+      <c r="C25" s="48"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="48"/>
+      <c r="F25" s="48"/>
+      <c r="G25" s="48"/>
+      <c r="H25" s="48"/>
+      <c r="I25" s="48"/>
+      <c r="J25" s="48"/>
+      <c r="K25" s="48"/>
+      <c r="L25" s="48"/>
     </row>
     <row r="26">
-      <c r="A26" s="49"/>
-      <c r="B26" s="49"/>
-      <c r="C26" s="49"/>
-      <c r="D26" s="49"/>
-      <c r="E26" s="49"/>
-      <c r="F26" s="49"/>
-      <c r="G26" s="49"/>
-      <c r="H26" s="49"/>
-      <c r="I26" s="49"/>
-      <c r="J26" s="49"/>
-      <c r="K26" s="49"/>
-      <c r="L26" s="49"/>
+      <c r="A26" s="48"/>
+      <c r="B26" s="48"/>
+      <c r="C26" s="48"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="48"/>
+      <c r="F26" s="48"/>
+      <c r="G26" s="48"/>
+      <c r="H26" s="48"/>
+      <c r="I26" s="48"/>
+      <c r="J26" s="48"/>
+      <c r="K26" s="48"/>
+      <c r="L26" s="48"/>
     </row>
     <row r="27">
-      <c r="A27" s="49"/>
-      <c r="B27" s="49"/>
-      <c r="C27" s="49"/>
-      <c r="D27" s="49"/>
-      <c r="E27" s="49"/>
-      <c r="F27" s="49"/>
-      <c r="G27" s="49"/>
-      <c r="H27" s="49"/>
-      <c r="I27" s="49"/>
-      <c r="J27" s="49"/>
-      <c r="K27" s="49"/>
-      <c r="L27" s="49"/>
+      <c r="A27" s="48"/>
+      <c r="B27" s="48"/>
+      <c r="C27" s="48"/>
+      <c r="D27" s="48"/>
+      <c r="E27" s="48"/>
+      <c r="F27" s="48"/>
+      <c r="G27" s="48"/>
+      <c r="H27" s="48"/>
+      <c r="I27" s="48"/>
+      <c r="J27" s="48"/>
+      <c r="K27" s="48"/>
+      <c r="L27" s="48"/>
     </row>
     <row r="28">
-      <c r="A28" s="49"/>
-      <c r="B28" s="49"/>
-      <c r="C28" s="49"/>
-      <c r="D28" s="49"/>
-      <c r="E28" s="49"/>
-      <c r="F28" s="49"/>
-      <c r="G28" s="49"/>
-      <c r="H28" s="49"/>
-      <c r="I28" s="49"/>
-      <c r="J28" s="49"/>
-      <c r="K28" s="49"/>
-      <c r="L28" s="49"/>
+      <c r="A28" s="48"/>
+      <c r="B28" s="48"/>
+      <c r="C28" s="48"/>
+      <c r="D28" s="48"/>
+      <c r="E28" s="48"/>
+      <c r="F28" s="48"/>
+      <c r="G28" s="48"/>
+      <c r="H28" s="48"/>
+      <c r="I28" s="48"/>
+      <c r="J28" s="48"/>
+      <c r="K28" s="48"/>
+      <c r="L28" s="48"/>
     </row>
     <row r="29">
-      <c r="A29" s="49"/>
-      <c r="B29" s="49"/>
-      <c r="C29" s="49"/>
-      <c r="D29" s="49"/>
-      <c r="E29" s="49"/>
-      <c r="F29" s="49"/>
-      <c r="G29" s="49"/>
-      <c r="H29" s="49"/>
-      <c r="I29" s="49"/>
-      <c r="J29" s="49"/>
-      <c r="K29" s="49"/>
-      <c r="L29" s="49"/>
+      <c r="A29" s="48"/>
+      <c r="B29" s="48"/>
+      <c r="C29" s="48"/>
+      <c r="D29" s="48"/>
+      <c r="E29" s="48"/>
+      <c r="F29" s="48"/>
+      <c r="G29" s="48"/>
+      <c r="H29" s="48"/>
+      <c r="I29" s="48"/>
+      <c r="J29" s="48"/>
+      <c r="K29" s="48"/>
+      <c r="L29" s="48"/>
     </row>
     <row r="30">
-      <c r="A30" s="49"/>
-      <c r="B30" s="49"/>
-      <c r="C30" s="49"/>
-      <c r="D30" s="49"/>
-      <c r="E30" s="49"/>
-      <c r="F30" s="49"/>
-      <c r="G30" s="49"/>
-      <c r="H30" s="49"/>
-      <c r="I30" s="49"/>
-      <c r="J30" s="49"/>
-      <c r="K30" s="49"/>
-      <c r="L30" s="49"/>
+      <c r="A30" s="48"/>
+      <c r="B30" s="48"/>
+      <c r="C30" s="48"/>
+      <c r="D30" s="48"/>
+      <c r="E30" s="48"/>
+      <c r="F30" s="48"/>
+      <c r="G30" s="48"/>
+      <c r="H30" s="48"/>
+      <c r="I30" s="48"/>
+      <c r="J30" s="48"/>
+      <c r="K30" s="48"/>
+      <c r="L30" s="48"/>
     </row>
     <row r="31">
-      <c r="A31" s="49"/>
-      <c r="B31" s="49"/>
-      <c r="C31" s="49"/>
-      <c r="D31" s="49"/>
-      <c r="E31" s="49"/>
-      <c r="F31" s="49"/>
-      <c r="G31" s="49"/>
-      <c r="H31" s="49"/>
-      <c r="I31" s="49"/>
-      <c r="J31" s="49"/>
-      <c r="K31" s="49"/>
-      <c r="L31" s="49"/>
+      <c r="A31" s="48"/>
+      <c r="B31" s="48"/>
+      <c r="C31" s="48"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="48"/>
+      <c r="F31" s="48"/>
+      <c r="G31" s="48"/>
+      <c r="H31" s="48"/>
+      <c r="I31" s="48"/>
+      <c r="J31" s="48"/>
+      <c r="K31" s="48"/>
+      <c r="L31" s="48"/>
     </row>
     <row r="32">
-      <c r="A32" s="49"/>
-      <c r="B32" s="49"/>
-      <c r="C32" s="49"/>
-      <c r="D32" s="49"/>
-      <c r="E32" s="49"/>
-      <c r="F32" s="49"/>
-      <c r="G32" s="49"/>
-      <c r="H32" s="49"/>
-      <c r="I32" s="49"/>
-      <c r="J32" s="49"/>
-      <c r="K32" s="49"/>
-      <c r="L32" s="49"/>
+      <c r="A32" s="48"/>
+      <c r="B32" s="48"/>
+      <c r="C32" s="48"/>
+      <c r="D32" s="48"/>
+      <c r="E32" s="48"/>
+      <c r="F32" s="48"/>
+      <c r="G32" s="48"/>
+      <c r="H32" s="48"/>
+      <c r="I32" s="48"/>
+      <c r="J32" s="48"/>
+      <c r="K32" s="48"/>
+      <c r="L32" s="48"/>
     </row>
     <row r="33">
-      <c r="A33" s="49"/>
-      <c r="B33" s="49"/>
-      <c r="C33" s="49"/>
-      <c r="D33" s="49"/>
-      <c r="E33" s="49"/>
-      <c r="F33" s="49"/>
-      <c r="G33" s="49"/>
-      <c r="H33" s="49"/>
-      <c r="I33" s="49"/>
-      <c r="J33" s="49"/>
-      <c r="K33" s="49"/>
-      <c r="L33" s="49"/>
+      <c r="A33" s="48"/>
+      <c r="B33" s="48"/>
+      <c r="C33" s="48"/>
+      <c r="D33" s="48"/>
+      <c r="E33" s="48"/>
+      <c r="F33" s="48"/>
+      <c r="G33" s="48"/>
+      <c r="H33" s="48"/>
+      <c r="I33" s="48"/>
+      <c r="J33" s="48"/>
+      <c r="K33" s="48"/>
+      <c r="L33" s="48"/>
     </row>
     <row r="34">
-      <c r="A34" s="49"/>
-      <c r="B34" s="49"/>
-      <c r="C34" s="49"/>
-      <c r="D34" s="49"/>
-      <c r="E34" s="49"/>
-      <c r="F34" s="49"/>
-      <c r="G34" s="49"/>
-      <c r="H34" s="49"/>
-      <c r="I34" s="49"/>
-      <c r="J34" s="49"/>
-      <c r="K34" s="49"/>
-      <c r="L34" s="49"/>
+      <c r="A34" s="48"/>
+      <c r="B34" s="48"/>
+      <c r="C34" s="48"/>
+      <c r="D34" s="48"/>
+      <c r="E34" s="48"/>
+      <c r="F34" s="48"/>
+      <c r="G34" s="48"/>
+      <c r="H34" s="48"/>
+      <c r="I34" s="48"/>
+      <c r="J34" s="48"/>
+      <c r="K34" s="48"/>
+      <c r="L34" s="48"/>
     </row>
     <row r="35">
-      <c r="A35" s="49"/>
-      <c r="B35" s="49"/>
-      <c r="C35" s="49"/>
-      <c r="D35" s="49"/>
-      <c r="E35" s="49"/>
-      <c r="F35" s="49"/>
-      <c r="G35" s="49"/>
-      <c r="H35" s="49"/>
-      <c r="I35" s="49"/>
-      <c r="J35" s="49"/>
-      <c r="K35" s="49"/>
-      <c r="L35" s="49"/>
+      <c r="A35" s="48"/>
+      <c r="B35" s="48"/>
+      <c r="C35" s="48"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="48"/>
+      <c r="F35" s="48"/>
+      <c r="G35" s="48"/>
+      <c r="H35" s="48"/>
+      <c r="I35" s="48"/>
+      <c r="J35" s="48"/>
+      <c r="K35" s="48"/>
+      <c r="L35" s="48"/>
     </row>
     <row r="36">
-      <c r="A36" s="49"/>
-      <c r="B36" s="49"/>
-      <c r="C36" s="49"/>
-      <c r="D36" s="49"/>
-      <c r="E36" s="49"/>
-      <c r="F36" s="49"/>
-      <c r="G36" s="49"/>
-      <c r="H36" s="49"/>
-      <c r="I36" s="49"/>
-      <c r="J36" s="49"/>
-      <c r="K36" s="49"/>
-      <c r="L36" s="49"/>
+      <c r="A36" s="48"/>
+      <c r="B36" s="48"/>
+      <c r="C36" s="48"/>
+      <c r="D36" s="48"/>
+      <c r="E36" s="48"/>
+      <c r="F36" s="48"/>
+      <c r="G36" s="48"/>
+      <c r="H36" s="48"/>
+      <c r="I36" s="48"/>
+      <c r="J36" s="48"/>
+      <c r="K36" s="48"/>
+      <c r="L36" s="48"/>
     </row>
     <row r="37">
-      <c r="A37" s="49"/>
-      <c r="B37" s="49"/>
-      <c r="C37" s="49"/>
-      <c r="D37" s="49"/>
-      <c r="E37" s="49"/>
-      <c r="F37" s="49"/>
-      <c r="G37" s="49"/>
-      <c r="H37" s="49"/>
-      <c r="I37" s="49"/>
-      <c r="J37" s="49"/>
-      <c r="K37" s="49"/>
-      <c r="L37" s="49"/>
+      <c r="A37" s="48"/>
+      <c r="B37" s="48"/>
+      <c r="C37" s="48"/>
+      <c r="D37" s="48"/>
+      <c r="E37" s="48"/>
+      <c r="F37" s="48"/>
+      <c r="G37" s="48"/>
+      <c r="H37" s="48"/>
+      <c r="I37" s="48"/>
+      <c r="J37" s="48"/>
+      <c r="K37" s="48"/>
+      <c r="L37" s="48"/>
     </row>
     <row r="38">
-      <c r="A38" s="49"/>
-      <c r="B38" s="49"/>
-      <c r="C38" s="49"/>
-      <c r="D38" s="49"/>
-      <c r="E38" s="49"/>
-      <c r="F38" s="49"/>
-      <c r="G38" s="49"/>
-      <c r="H38" s="49"/>
-      <c r="I38" s="49"/>
-      <c r="J38" s="49"/>
-      <c r="K38" s="49"/>
-      <c r="L38" s="49"/>
+      <c r="A38" s="48"/>
+      <c r="B38" s="48"/>
+      <c r="C38" s="48"/>
+      <c r="D38" s="48"/>
+      <c r="E38" s="48"/>
+      <c r="F38" s="48"/>
+      <c r="G38" s="48"/>
+      <c r="H38" s="48"/>
+      <c r="I38" s="48"/>
+      <c r="J38" s="48"/>
+      <c r="K38" s="48"/>
+      <c r="L38" s="48"/>
     </row>
     <row r="39">
-      <c r="A39" s="49"/>
-      <c r="B39" s="49"/>
-      <c r="C39" s="49"/>
-      <c r="D39" s="49"/>
-      <c r="E39" s="49"/>
-      <c r="F39" s="49"/>
-      <c r="G39" s="49"/>
-      <c r="H39" s="49"/>
-      <c r="I39" s="49"/>
-      <c r="J39" s="49"/>
-      <c r="K39" s="49"/>
-      <c r="L39" s="49"/>
+      <c r="A39" s="48"/>
+      <c r="B39" s="48"/>
+      <c r="C39" s="48"/>
+      <c r="D39" s="48"/>
+      <c r="E39" s="48"/>
+      <c r="F39" s="48"/>
+      <c r="G39" s="48"/>
+      <c r="H39" s="48"/>
+      <c r="I39" s="48"/>
+      <c r="J39" s="48"/>
+      <c r="K39" s="48"/>
+      <c r="L39" s="48"/>
     </row>
     <row r="40">
-      <c r="A40" s="49"/>
-      <c r="B40" s="49"/>
-      <c r="C40" s="49"/>
-      <c r="D40" s="49"/>
-      <c r="E40" s="49"/>
-      <c r="F40" s="49"/>
-      <c r="G40" s="49"/>
-      <c r="H40" s="49"/>
-      <c r="I40" s="49"/>
-      <c r="J40" s="49"/>
-      <c r="K40" s="49"/>
-      <c r="L40" s="49"/>
+      <c r="A40" s="48"/>
+      <c r="B40" s="48"/>
+      <c r="C40" s="48"/>
+      <c r="D40" s="48"/>
+      <c r="E40" s="48"/>
+      <c r="F40" s="48"/>
+      <c r="G40" s="48"/>
+      <c r="H40" s="48"/>
+      <c r="I40" s="48"/>
+      <c r="J40" s="48"/>
+      <c r="K40" s="48"/>
+      <c r="L40" s="48"/>
     </row>
     <row r="41">
-      <c r="A41" s="49"/>
-      <c r="B41" s="49"/>
-      <c r="C41" s="49"/>
-      <c r="D41" s="49"/>
-      <c r="E41" s="49"/>
-      <c r="F41" s="49"/>
-      <c r="G41" s="49"/>
-      <c r="H41" s="49"/>
-      <c r="I41" s="49"/>
-      <c r="J41" s="49"/>
-      <c r="K41" s="49"/>
-      <c r="L41" s="49"/>
+      <c r="A41" s="48"/>
+      <c r="B41" s="48"/>
+      <c r="C41" s="48"/>
+      <c r="D41" s="48"/>
+      <c r="E41" s="48"/>
+      <c r="F41" s="48"/>
+      <c r="G41" s="48"/>
+      <c r="H41" s="48"/>
+      <c r="I41" s="48"/>
+      <c r="J41" s="48"/>
+      <c r="K41" s="48"/>
+      <c r="L41" s="48"/>
     </row>
     <row r="42">
-      <c r="A42" s="49"/>
-      <c r="B42" s="49"/>
-      <c r="C42" s="49"/>
-      <c r="D42" s="49"/>
-      <c r="E42" s="49"/>
-      <c r="F42" s="49"/>
-      <c r="G42" s="49"/>
-      <c r="H42" s="49"/>
-      <c r="I42" s="49"/>
-      <c r="J42" s="49"/>
-      <c r="K42" s="49"/>
-      <c r="L42" s="49"/>
+      <c r="A42" s="48"/>
+      <c r="B42" s="48"/>
+      <c r="C42" s="48"/>
+      <c r="D42" s="48"/>
+      <c r="E42" s="48"/>
+      <c r="F42" s="48"/>
+      <c r="G42" s="48"/>
+      <c r="H42" s="48"/>
+      <c r="I42" s="48"/>
+      <c r="J42" s="48"/>
+      <c r="K42" s="48"/>
+      <c r="L42" s="48"/>
     </row>
     <row r="43">
-      <c r="A43" s="49"/>
-      <c r="B43" s="49"/>
-      <c r="C43" s="49"/>
-      <c r="D43" s="49"/>
-      <c r="E43" s="49"/>
-      <c r="F43" s="49"/>
-      <c r="G43" s="49"/>
-      <c r="H43" s="49"/>
-      <c r="I43" s="49"/>
-      <c r="J43" s="49"/>
-      <c r="K43" s="49"/>
-      <c r="L43" s="49"/>
+      <c r="A43" s="48"/>
+      <c r="B43" s="48"/>
+      <c r="C43" s="48"/>
+      <c r="D43" s="48"/>
+      <c r="E43" s="48"/>
+      <c r="F43" s="48"/>
+      <c r="G43" s="48"/>
+      <c r="H43" s="48"/>
+      <c r="I43" s="48"/>
+      <c r="J43" s="48"/>
+      <c r="K43" s="48"/>
+      <c r="L43" s="48"/>
     </row>
     <row r="44">
-      <c r="A44" s="49"/>
-      <c r="B44" s="49"/>
-      <c r="C44" s="49"/>
-      <c r="D44" s="49"/>
-      <c r="E44" s="49"/>
-      <c r="F44" s="49"/>
-      <c r="G44" s="49"/>
-      <c r="H44" s="49"/>
-      <c r="I44" s="49"/>
-      <c r="J44" s="49"/>
-      <c r="K44" s="49"/>
-      <c r="L44" s="49"/>
+      <c r="A44" s="48"/>
+      <c r="B44" s="48"/>
+      <c r="C44" s="48"/>
+      <c r="D44" s="48"/>
+      <c r="E44" s="48"/>
+      <c r="F44" s="48"/>
+      <c r="G44" s="48"/>
+      <c r="H44" s="48"/>
+      <c r="I44" s="48"/>
+      <c r="J44" s="48"/>
+      <c r="K44" s="48"/>
+      <c r="L44" s="48"/>
     </row>
     <row r="45">
-      <c r="A45" s="49"/>
-      <c r="B45" s="49"/>
-      <c r="C45" s="49"/>
-      <c r="D45" s="49"/>
-      <c r="E45" s="49"/>
-      <c r="F45" s="49"/>
-      <c r="G45" s="49"/>
-      <c r="H45" s="49"/>
-      <c r="I45" s="49"/>
-      <c r="J45" s="49"/>
-      <c r="K45" s="49"/>
-      <c r="L45" s="49"/>
+      <c r="A45" s="48"/>
+      <c r="B45" s="48"/>
+      <c r="C45" s="48"/>
+      <c r="D45" s="48"/>
+      <c r="E45" s="48"/>
+      <c r="F45" s="48"/>
+      <c r="G45" s="48"/>
+      <c r="H45" s="48"/>
+      <c r="I45" s="48"/>
+      <c r="J45" s="48"/>
+      <c r="K45" s="48"/>
+      <c r="L45" s="48"/>
     </row>
     <row r="46">
-      <c r="A46" s="49"/>
-      <c r="B46" s="49"/>
-      <c r="C46" s="49"/>
-      <c r="D46" s="49"/>
-      <c r="E46" s="49"/>
-      <c r="F46" s="49"/>
-      <c r="G46" s="49"/>
-      <c r="H46" s="49"/>
-      <c r="I46" s="49"/>
-      <c r="J46" s="49"/>
-      <c r="K46" s="49"/>
-      <c r="L46" s="49"/>
+      <c r="A46" s="48"/>
+      <c r="B46" s="48"/>
+      <c r="C46" s="48"/>
+      <c r="D46" s="48"/>
+      <c r="E46" s="48"/>
+      <c r="F46" s="48"/>
+      <c r="G46" s="48"/>
+      <c r="H46" s="48"/>
+      <c r="I46" s="48"/>
+      <c r="J46" s="48"/>
+      <c r="K46" s="48"/>
+      <c r="L46" s="48"/>
     </row>
     <row r="47">
-      <c r="A47" s="49"/>
-      <c r="B47" s="49"/>
-      <c r="C47" s="49"/>
-      <c r="D47" s="49"/>
-      <c r="E47" s="49"/>
-      <c r="F47" s="49"/>
-      <c r="G47" s="49"/>
-      <c r="H47" s="49"/>
-      <c r="I47" s="49"/>
-      <c r="J47" s="49"/>
-      <c r="K47" s="49"/>
-      <c r="L47" s="49"/>
+      <c r="A47" s="48"/>
+      <c r="B47" s="48"/>
+      <c r="C47" s="48"/>
+      <c r="D47" s="48"/>
+      <c r="E47" s="48"/>
+      <c r="F47" s="48"/>
+      <c r="G47" s="48"/>
+      <c r="H47" s="48"/>
+      <c r="I47" s="48"/>
+      <c r="J47" s="48"/>
+      <c r="K47" s="48"/>
+      <c r="L47" s="48"/>
     </row>
     <row r="48">
-      <c r="A48" s="49"/>
-      <c r="B48" s="49"/>
-      <c r="C48" s="49"/>
-      <c r="D48" s="49"/>
-      <c r="E48" s="49"/>
-      <c r="F48" s="49"/>
-      <c r="G48" s="49"/>
-      <c r="H48" s="49"/>
-      <c r="I48" s="49"/>
-      <c r="J48" s="49"/>
-      <c r="K48" s="49"/>
-      <c r="L48" s="49"/>
+      <c r="A48" s="48"/>
+      <c r="B48" s="48"/>
+      <c r="C48" s="48"/>
+      <c r="D48" s="48"/>
+      <c r="E48" s="48"/>
+      <c r="F48" s="48"/>
+      <c r="G48" s="48"/>
+      <c r="H48" s="48"/>
+      <c r="I48" s="48"/>
+      <c r="J48" s="48"/>
+      <c r="K48" s="48"/>
+      <c r="L48" s="48"/>
     </row>
     <row r="49">
-      <c r="A49" s="49"/>
-      <c r="B49" s="49"/>
-      <c r="C49" s="49"/>
-      <c r="D49" s="49"/>
-      <c r="E49" s="49"/>
-      <c r="F49" s="49"/>
-      <c r="G49" s="49"/>
-      <c r="H49" s="49"/>
-      <c r="I49" s="49"/>
-      <c r="J49" s="49"/>
-      <c r="K49" s="49"/>
-      <c r="L49" s="49"/>
+      <c r="A49" s="48"/>
+      <c r="B49" s="48"/>
+      <c r="C49" s="48"/>
+      <c r="D49" s="48"/>
+      <c r="E49" s="48"/>
+      <c r="F49" s="48"/>
+      <c r="G49" s="48"/>
+      <c r="H49" s="48"/>
+      <c r="I49" s="48"/>
+      <c r="J49" s="48"/>
+      <c r="K49" s="48"/>
+      <c r="L49" s="48"/>
     </row>
     <row r="50">
-      <c r="A50" s="49"/>
-      <c r="B50" s="49"/>
-      <c r="C50" s="49"/>
-      <c r="D50" s="49"/>
-      <c r="E50" s="49"/>
-      <c r="F50" s="49"/>
-      <c r="G50" s="49"/>
-      <c r="H50" s="49"/>
-      <c r="I50" s="49"/>
-      <c r="J50" s="49"/>
-      <c r="K50" s="49"/>
-      <c r="L50" s="49"/>
+      <c r="A50" s="48"/>
+      <c r="B50" s="48"/>
+      <c r="C50" s="48"/>
+      <c r="D50" s="48"/>
+      <c r="E50" s="48"/>
+      <c r="F50" s="48"/>
+      <c r="G50" s="48"/>
+      <c r="H50" s="48"/>
+      <c r="I50" s="48"/>
+      <c r="J50" s="48"/>
+      <c r="K50" s="48"/>
+      <c r="L50" s="48"/>
     </row>
     <row r="51">
-      <c r="A51" s="49"/>
-      <c r="B51" s="49"/>
-      <c r="C51" s="49"/>
-      <c r="D51" s="49"/>
-      <c r="E51" s="49"/>
-      <c r="F51" s="49"/>
-      <c r="G51" s="49"/>
-      <c r="H51" s="49"/>
-      <c r="I51" s="49"/>
-      <c r="J51" s="49"/>
-      <c r="K51" s="49"/>
-      <c r="L51" s="49"/>
+      <c r="A51" s="48"/>
+      <c r="B51" s="48"/>
+      <c r="C51" s="48"/>
+      <c r="D51" s="48"/>
+      <c r="E51" s="48"/>
+      <c r="F51" s="48"/>
+      <c r="G51" s="48"/>
+      <c r="H51" s="48"/>
+      <c r="I51" s="48"/>
+      <c r="J51" s="48"/>
+      <c r="K51" s="48"/>
+      <c r="L51" s="48"/>
     </row>
     <row r="52">
-      <c r="A52" s="50"/>
-      <c r="B52" s="50"/>
-      <c r="C52" s="50"/>
-      <c r="D52" s="50"/>
-      <c r="E52" s="50"/>
-      <c r="F52" s="50"/>
-      <c r="G52" s="50"/>
-      <c r="H52" s="50"/>
-      <c r="I52" s="50"/>
-      <c r="J52" s="50"/>
-      <c r="K52" s="50"/>
-      <c r="L52" s="50"/>
+      <c r="A52" s="48"/>
+      <c r="B52" s="48"/>
+      <c r="C52" s="48"/>
+      <c r="D52" s="48"/>
+      <c r="E52" s="48"/>
+      <c r="F52" s="48"/>
+      <c r="G52" s="48"/>
+      <c r="H52" s="48"/>
+      <c r="I52" s="48"/>
+      <c r="J52" s="48"/>
+      <c r="K52" s="48"/>
+      <c r="L52" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
style(vehicle-export): center all data cells; fix Pelawat title font
Title + headers were already centered; added horizontal="center" to each
template's data-cell style so every column and row is centered (template +
byte-cloned export). Also restored the <family> hint on Pelawat's title font
(it had been dropped when that template was generated), so its title renders
like the others. Direct styles.xml edits — fonts otherwise untouched.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/Kontraktor.xlsx
+++ b/assets/templates/Kontraktor.xlsx
@@ -516,7 +516,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf applyAlignment="1" numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>

</xml_diff>